<commit_message>
Expand onboarding template's step guide with 3 previously-missed steps
Adds explicit steps for the three gotchas hit onboarding Ram Krishna
Banquet, each as its own numbered row rather than a buried parenthetical:
(1) deciding the hosting URL and knowing a custom subdomain needs a
secondary Hosting site, (2) verifying the service account is created in
the SAME project as the web app config — the exact mismatch that blocked
the first deploy attempt, and (3) opening Firestore rules after the first
deploy, flagged as REQUIRED since a fresh "production mode" database
silently denies all reads/writes with no visible error otherwise.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/venue-onboarding-template.xlsx
+++ b/templates/venue-onboarding-template.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="61">
   <si>
     <t>Status</t>
   </si>
@@ -147,13 +147,19 @@
     <t>Create the Firebase project</t>
   </si>
   <si>
-    <t>Click "Add project", name it (e.g. "My Venue Banquet"), Analytics is optional (fine to disable), click Create. Wait for provisioning to finish.</t>
+    <t>Click "Add project", name it (e.g. "My Venue Banquet"), Analytics is optional (fine to disable), click Create. Wait for provisioning to finish. Note the exact project ID shown (auto-generated from the name, sometimes with a random suffix) — every later step must use THIS SAME project ID, see Step 6.</t>
   </si>
   <si>
     <t>Create the Firestore database</t>
   </si>
   <si>
-    <t>Left nav: Build &gt; Firestore Database &gt; Create database. Choose "Start in production mode". Pick a region NOW — this cannot be changed later without deleting and recreating the database. Click Enable. NOTE: "production mode" defaults to deny-all security rules — the app will silently fall back to local-only storage (no visible error) until those rules are explicitly opened after the first deploy. onboard-venue.js's printed next-steps cover this; don't skip that step.</t>
+    <t>Left nav: Build &gt; Firestore Database &gt; Create database. Choose "Start in production mode". Pick a region NOW — this cannot be changed later without deleting and recreating the database. Click Enable.</t>
+  </si>
+  <si>
+    <t>Decide the hosting URL</t>
+  </si>
+  <si>
+    <t>Default (simplest, zero extra setup): &lt;projectId&gt;.web.app — always available automatically. If you'd rather have a different/nicer subdomain (e.g. "myvenue.web.app" instead of "myvenue-a8f21.web.app"), that's fine and supported, but it requires creating a SECOND Hosting site inside this project — onboard-venue.js detects this from the "Hosting URL (host)" column and prints the exact one-time site-creation command as part of its next-steps output. Just be aware it's an extra step, not a bug, if your requested host doesn't match the project's default.</t>
   </si>
   <si>
     <t>Register a Web App and copy its config</t>
@@ -162,10 +168,10 @@
     <t>Left nav: Project settings (gear icon) &gt; General tab &gt; scroll to "Your apps" &gt; click the &lt;/&gt; (Web) icon &gt; give it a nickname &gt; Register app. Firebase Hosting setup in this wizard can be skipped/ignored. Copy the six values shown in the firebaseConfig block (apiKey, authDomain, projectId, storageBucket, messagingSenderId, appId) into the matching columns on the "New Venues" sheet.</t>
   </si>
   <si>
-    <t>Create a service account for deploys</t>
-  </si>
-  <si>
-    <t>Go to https://console.cloud.google.com/iam-admin/serviceaccounts and make sure the new Firebase project is selected (top dropdown). Click "Create Service Account", name it e.g. "deploy-bot", click Create and Continue.</t>
+    <t>Create a service account for deploys — SAME PROJECT ONLY</t>
+  </si>
+  <si>
+    <t>Go to https://console.cloud.google.com/iam-admin/serviceaccounts and check the project selector at the top says the EXACT project ID from Step 2/4 — not a similarly-named one, not a leftover from a previous attempt. (Real incident: a service account was created in the wrong project once, its key silently couldn't deploy anything for the venue it was meant for, and it wasn't caught until the deploy failed. Firebase project IDs are immutable and can't be aliased, so a mismatch here has no easy fix later — just recreate the key in the right project.) Click "Create Service Account", name it e.g. "deploy-bot", click Create and Continue.</t>
   </si>
   <si>
     <t>Grant it the Owner role</t>
@@ -177,13 +183,19 @@
     <t>Download the JSON key</t>
   </si>
   <si>
-    <t>Open the new service account &gt; Keys tab &gt; Add Key &gt; Create new key &gt; JSON &gt; it downloads automatically. Move that file to C:\Users\&lt;you&gt;\.banquet-credentials\&lt;projectId&gt;-service-account.json (create the folder if needed) — NEVER inside the git repo. Only fill in the "Service account key path" column on the New Venues sheet if you saved it somewhere else.</t>
+    <t>Open the new service account &gt; Keys tab &gt; Add Key &gt; Create new key &gt; JSON &gt; it downloads automatically. Move that file to C:\Users\&lt;you&gt;\.banquet-credentials\&lt;projectId&gt;-service-account.json (create the folder if needed) — NEVER inside the git repo. Only fill in the "Service account key path" column on the New Venues sheet if you saved it somewhere else. Sanity check before moving on: open the JSON and confirm its "project_id" field matches Step 2/4's project ID exactly.</t>
   </si>
   <si>
     <t>Fill in the New Venues row and hand the file back</t>
   </si>
   <si>
     <t>Fill in Status="Pending" and every column on one row of the "New Venues" sheet using what you collected above, save the file, and give it back (path or attachment) so the repo-side onboarding + first deploy can be run against it.</t>
+  </si>
+  <si>
+    <t>After the first deploy: open the Firestore rules — REQUIRED</t>
+  </si>
+  <si>
+    <t>"Production mode" (Step 3) defaults to deny-all security rules. Without this step the app deploys fine and LOOKS like it's working, but every read/write silently fails and it falls back to local-only storage in the browser — no visible error, easy to miss. This isn't optional or something to "decide on later" — it's required for the app to function at all. onboard-venue.js's printed next-steps include the exact commands (PowerShell, using the service account from Steps 6-8) to open this and a curl command to verify it actually took effect before trusting the app.</t>
   </si>
 </sst>
 </file>
@@ -888,7 +900,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -995,6 +1007,28 @@
         <v>56</v>
       </c>
     </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="4">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="4">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>